<commit_message>
Correct Coin #2 year to 1947
User verified against the physical coin (previously read as 1974).
</commit_message>
<xml_diff>
--- a/output/Austrian_Coin_Collection.xlsx
+++ b/output/Austrian_Coin_Collection.xlsx
@@ -291,7 +291,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1974</t>
+          <t xml:space="preserve">1947</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -316,7 +316,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date read as 1974 from vertical 19.74-style date split - moderate-high confidence</t>
+          <t xml:space="preserve">Confirmed by user - first year of this 1 Groschen type</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Coin #3 year to 1968
User verified against the physical coin (previously read as 1967).
</commit_message>
<xml_diff>
--- a/output/Austrian_Coin_Collection.xlsx
+++ b/output/Austrian_Coin_Collection.xlsx
@@ -338,7 +338,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1967</t>
+          <t xml:space="preserve">1968</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -358,12 +358,12 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle, REPUBLIK OSTERREICH, partial date 67 visible beneath tail feathers. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same design/wear family as Coin 1.</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle, REPUBLIK OSTERREICH, partial date visible beneath tail feathers. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same design/wear family as Coin 1.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last two digits (67) fairly clear; 19-prefix inferred, not directly visible - moderate confidence</t>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply user verification corrections to coin catalog
Coins #6, #9, #13, #14, #17 corrected against physical coins:
- #6: 1969 -> 1966
- #9: 1961 -> 1947
- #13: 1975 -> 1973
- #14: 2 Groschen 1984 -> 10 Groschen 1948 (zinc)
- #17: 1961 -> 1947
</commit_message>
<xml_diff>
--- a/output/Austrian_Coin_Collection.xlsx
+++ b/output/Austrian_Coin_Collection.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1969</t>
+          <t xml:space="preserve">1966</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -499,12 +499,12 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate corrosion/pitting similar to Coins 1/3/4.</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate corrosion/pitting similar to Coins 1/3/4. Same year as Coins 12/20 - duplicate.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence on date - clear vertical digits</t>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1961</t>
+          <t xml:space="preserve">1947</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -640,12 +640,12 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Darker/duller surface than Coin 2, more visible wear.</t>
+          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Darker/duller surface than Coin 2, more visible wear. Same year as Coin 2 - duplicate.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date cluster cramped/worn - moderate confidence only</t>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1975</t>
+          <t xml:space="preserve">1973</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs.</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coins 1/4 - duplicate.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence - date clear</t>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 Groschen</t>
+          <t xml:space="preserve">10 Groschen</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1984</t>
+          <t xml:space="preserve">1948</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aluminum</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large angular 2, GROSCHEN, edelweiss sprigs.</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large angular 2-digit 10, GROSCHEN, edelweiss sprigs.</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Digit cluster tightly packed - moderate confidence on date</t>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1961</t>
+          <t xml:space="preserve">1947</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1016,12 +1016,12 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Similar toning/wear to Coin 9 - possible duplicate year.</t>
+          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Similar toning/wear to Coin 9 - same year as Coins 2/9, duplicate.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tail digits (61) reasonably clear - moderate confidence overall</t>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>
@@ -1198,11 +1198,11 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 Groschen count</t>
+          <t xml:space="preserve">10 Groschen count</t>
         </is>
       </c>
       <c r="B30" s="9">
-        <f>COUNTIF(B5:B24,"2 Groschen")</f>
+        <f>COUNTIF(B5:B24,"10 Groschen")</f>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Remove 4 duplicate coins per user decision, renumber 1-16
Removed original coins #3, #4, #6, #17 (worse-graded member of each
3-of-a-kind duplicate group, per user's in-hand comparison). Remaining
16 coins renumbered sequentially; new "Orig. #" column preserves each
coin's original catalog number for traceability. Dropped the now-stale
pre-decision duplicates reference doc.
</commit_message>
<xml_diff>
--- a/output/Austrian_Coin_Collection.xlsx
+++ b/output/Austrian_Coin_Collection.xlsx
@@ -139,14 +139,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="60" customWidth="1"/>
-    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="60" customWidth="1"/>
+    <col min="10" max="10" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -163,6 +164,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -178,6 +180,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -187,40 +190,45 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Orig. #</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Denomination</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Country</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Year</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mint</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Composition</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Grade (est.)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Confidence Flags</t>
         </is>
@@ -234,40 +242,45 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1973</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Surface shows zinc corrosion/porosity typical of the composition/era.</t>
-        </is>
-      </c>
       <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Surface shows zinc corrosion/porosity typical of the composition/era. Kept over original Coin 4 (same year/grade) - user preferred this one's appearance.</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -281,40 +294,45 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1 Groschen</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1947</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Aluminum</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">XF-AU (photo estimate)</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Bright aluminum surface, minimal wear, crisp legends.</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user - first year of this 1 Groschen type</t>
         </is>
@@ -328,42 +346,47 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1968</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1976</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle, REPUBLIK OSTERREICH, partial date visible beneath tail feathers. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same design/wear family as Coin 1.</t>
+          <t xml:space="preserve">XF (photo estimate)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirmed by user</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Sharper/cleaner surfaces than most others in the collection, minimal corrosion, crisp legends.</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - photo sharp and well-lit</t>
         </is>
       </c>
     </row>
@@ -375,42 +398,47 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1973</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1980</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Duplicate denomination/year of Coin 1 - confirmed by user as a separate physical coin, not a resubmitted photo.</t>
+          <t xml:space="preserve">AU (photo estimate)</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date read as 1973 - same confidence basis as Coin 1</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Sharp strike, crisp feather detail, minimal wear.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - date and design very clear</t>
         </is>
       </c>
     </row>
@@ -422,42 +450,47 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1976</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1965</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">XF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Sharper/cleaner surfaces than Coins 1/3/4, minimal corrosion, crisp legends.</t>
+          <t xml:space="preserve">XF-AU (photo estimate)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence - photo sharp and well-lit</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp strike, good detail, light wear.</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - date very clear</t>
         </is>
       </c>
     </row>
@@ -469,40 +502,45 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">1 Groschen</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1966</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1947</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VF (photo estimate)</t>
+          <t xml:space="preserve">Aluminum</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate corrosion/pitting similar to Coins 1/3/4. Same year as Coins 12/20 - duplicate.</t>
+          <t xml:space="preserve">F-VF (photo estimate)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Darker/duller surface than Coin 2, more visible wear. Kept over original Coin 17 (same year/grade) - user preferred this one's appearance.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -516,42 +554,47 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1980</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1982</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">AU (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Sharp strike, crisp feather detail, minimal wear.</t>
+          <t xml:space="preserve">XF-AU (photo estimate)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence - date and design very clear</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp strike, good detail.</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - date very clear</t>
         </is>
       </c>
     </row>
@@ -563,42 +606,47 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1965</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1977</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">XF-AU (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp strike, good detail, light wear.</t>
+          <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence - date very clear</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate wear, legends fully legible.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - date clear</t>
         </is>
       </c>
     </row>
@@ -610,40 +658,45 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 Groschen</t>
+          <t xml:space="preserve">12</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1947</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1966</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aluminum</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">F-VF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Darker/duller surface than Coin 2, more visible wear. Same year as Coin 2 - duplicate.</t>
+          <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate wear, legends clear. Kept over original Coin 6 (same year/grade) - user felt this coin looks smoother and less rough.</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -657,42 +710,47 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">13</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1982</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1973</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">XF-AU (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp strike, good detail.</t>
+          <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence - date very clear</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 1 - duplicate, kept for its better grade.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>
@@ -704,42 +762,47 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">14</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">10 Groschen</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1977</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1948</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VF-XF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate wear, legends fully legible.</t>
+          <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence - date clear</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large angular 2-digit 10, GROSCHEN, edelweiss sprigs.</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed by user</t>
         </is>
       </c>
     </row>
@@ -751,42 +814,47 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">15</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1966</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1970</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate wear, legends clear.</t>
-        </is>
-      </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate-high confidence on date</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH (obverse photo has some motion blur). Reverse: large 5, GROSCHEN, edelweiss sprigs.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence on date - reverse sharp</t>
         </is>
       </c>
     </row>
@@ -798,42 +866,47 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">16</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1973</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1968</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VF-XF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coins 1/4 - duplicate.</t>
+          <t xml:space="preserve">XF (photo estimate)</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirmed by user</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp lettering, good detail. Kept over original Coin 3 (same year, lower grade).</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - date clear</t>
         </is>
       </c>
     </row>
@@ -845,42 +918,47 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">10 Groschen</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1948</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1968</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large angular 2-digit 10, GROSCHEN, edelweiss sprigs.</t>
+          <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirmed by user</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 13 - duplicate, kept for its grade.</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - date clear</t>
         </is>
       </c>
     </row>
@@ -892,42 +970,47 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">19</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1970</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VF (photo estimate)</t>
+          <t xml:space="preserve">Zinc</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH (obverse photo has some motion blur). Reverse: large 5, GROSCHEN, edelweiss sprigs.</t>
+          <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">High confidence on date - reverse sharp</t>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 12 - duplicate, both kept per user (not excessive).</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High confidence - date very clear</t>
         </is>
       </c>
     </row>
@@ -939,307 +1022,124 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen</t>
+          <t xml:space="preserve">20</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
+          <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1968</t>
+          <t xml:space="preserve">Austria (Second Republic)</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+          <t xml:space="preserve">1966</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">XF (photo estimate)</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp lettering, good detail.</t>
-        </is>
-      </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 9 - duplicate, kept as best grade in that group. Crisp detail.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">High confidence - date clear</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="70" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1 Groschen</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1947</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aluminum</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F-VF (photo estimate)</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Similar toning/wear to Coin 9 - same year as Coins 2/9, duplicate.</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confirmed by user</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="70" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Groschen</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1968</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Zinc</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VF-XF (photo estimate)</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same date as Coin 16 - duplicate year.</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">High confidence - date clear</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="70" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Groschen</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1970</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Zinc</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VF-XF (photo estimate)</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same date as Coin 15 - duplicate year.</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">High confidence - date very clear</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="70" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Groschen</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1966</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Zinc</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">XF (photo estimate)</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same date as Coin 12 - duplicate year. Crisp detail.</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">High confidence - date clear</t>
-        </is>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Collection Summary</t>
+        </is>
+      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total coins</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>COUNTA(A5:A20)</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Groschen count</t>
+        </is>
+      </c>
+      <c r="B25" s="9">
+        <f>COUNTIF(C5:C20,"5 Groschen")</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10 Groschen count</t>
+        </is>
+      </c>
+      <c r="B26" s="9">
+        <f>COUNTIF(C5:C20,"10 Groschen")</f>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collection Summary</t>
-        </is>
-      </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 Groschen count</t>
+        </is>
+      </c>
+      <c r="B27" s="9">
+        <f>COUNTIF(C5:C20,"1 Groschen")</f>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total coins</t>
+          <t xml:space="preserve">Earliest year</t>
         </is>
       </c>
       <c r="B28" s="9">
-        <f>COUNTA(A5:A24)</f>
+        <f>MIN(E5:E20)</f>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Groschen count</t>
+          <t xml:space="preserve">Latest year</t>
         </is>
       </c>
       <c r="B29" s="9">
-        <f>COUNTIF(B5:B24,"5 Groschen")</f>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10 Groschen count</t>
-        </is>
-      </c>
-      <c r="B30" s="9">
-        <f>COUNTIF(B5:B24,"10 Groschen")</f>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1 Groschen count</t>
-        </is>
-      </c>
-      <c r="B31" s="9">
-        <f>COUNTIF(B5:B24,"1 Groschen")</f>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Earliest year</t>
-        </is>
-      </c>
-      <c r="B32" s="9">
-        <f>MIN(D5:D24)</f>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Latest year</t>
-        </is>
-      </c>
-      <c r="B33" s="9">
-        <f>MAX(D5:D24)</f>
+        <f>MAX(E5:E20)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A23:C23"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Assign real Savoca invoice Coin IDs (SVCA-080..095), update tag design
- Added "Coin ID" column to the catalog (xlsx + docx), populated from the
  Savoca Blue Auction Invoice 68734, Lot 1136 ("Austria: lot of ca. 20
  coins"), continuing that invoice's SVCA numbering from its previous
  high (SVCA-079).
- Redesigned coin tags to match the user's reference tag standard: real
  Coin ID (orange), authority (navy), denom/date + mint + composition
  (dark gray), grade + lot receipt (teal italic), auction/year footer
  (small gray).
- Filled in Lot 1136's 20 item rows in the invoice spreadsheet: the 16
  kept coins get their real descriptions/grades/Coin IDs, the 4 removed
  duplicates (original #3, #4, #6, #17) are marked "duplicate" under
  Coin ID, all other invoice content left byte-identical.
</commit_message>
<xml_diff>
--- a/output/Austrian_Coin_Collection.xlsx
+++ b/output/Austrian_Coin_Collection.xlsx
@@ -139,15 +139,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="34" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="55" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -165,6 +166,7 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -181,6 +183,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -190,45 +193,50 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Coin ID</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Orig. #</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Denomination</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Country</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Year</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mint</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Composition</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Grade (est.)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Confidence Flags</t>
         </is>
@@ -242,45 +250,50 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-080</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1973</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Surface shows zinc corrosion/porosity typical of the composition/era. Kept over original Coin 4 (same year/grade) - user preferred this one's appearance.</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -294,45 +307,50 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-081</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">2</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">1 Groschen</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1947</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Aluminum</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">XF-AU (photo estimate)</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Bright aluminum surface, minimal wear, crisp legends.</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user - first year of this 1 Groschen type</t>
         </is>
@@ -346,45 +364,50 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-082</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">5</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1976</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">XF (photo estimate)</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Sharper/cleaner surfaces than most others in the collection, minimal corrosion, crisp legends.</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - photo sharp and well-lit</t>
         </is>
@@ -398,45 +421,50 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-083</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">7</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1980</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">AU (photo estimate)</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Sharp strike, crisp feather detail, minimal wear.</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date and design very clear</t>
         </is>
@@ -450,45 +478,50 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-084</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">8</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1965</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">XF-AU (photo estimate)</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp strike, good detail, light wear.</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date very clear</t>
         </is>
@@ -502,45 +535,50 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-085</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">9</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">1 Groschen</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1947</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Aluminum</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">F-VF (photo estimate)</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian eagle, REPUBLIK OSTERREICH. Reverse: large 1, GROSCHEN. Darker/duller surface than Coin 2, more visible wear. Kept over original Coin 17 (same year/grade) - user preferred this one's appearance.</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -554,45 +592,50 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-086</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">10</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1982</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">XF-AU (photo estimate)</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp strike, good detail.</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date very clear</t>
         </is>
@@ -606,45 +649,50 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-087</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">11</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1977</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate wear, legends fully legible.</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date clear</t>
         </is>
@@ -658,45 +706,50 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-088</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">12</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1966</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Moderate wear, legends clear. Kept over original Coin 6 (same year/grade) - user felt this coin looks smoother and less rough.</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -710,45 +763,50 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-089</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">13</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1973</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 1 - duplicate, kept for its better grade.</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -762,45 +820,50 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-090</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">14</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">10 Groschen</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1948</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large angular 2-digit 10, GROSCHEN, edelweiss sprigs.</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed by user</t>
         </is>
@@ -814,45 +877,50 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-091</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">15</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1970</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF (photo estimate)</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH (obverse photo has some motion blur). Reverse: large 5, GROSCHEN, edelweiss sprigs.</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence on date - reverse sharp</t>
         </is>
@@ -866,45 +934,50 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-092</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">16</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1968</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">XF (photo estimate)</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Crisp lettering, good detail. Kept over original Coin 3 (same year, lower grade).</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date clear</t>
         </is>
@@ -918,45 +991,50 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-093</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1968</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 13 - duplicate, kept for its grade.</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date clear</t>
         </is>
@@ -970,45 +1048,50 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-094</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">19</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">1970</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">VF-XF (photo estimate)</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 12 - duplicate, both kept per user (not excessive).</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date very clear</t>
         </is>
@@ -1022,45 +1105,50 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">COIN-2026-SVCA-095</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">20</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Groschen</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Austria (Second Republic)</t>
-        </is>
-      </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Austria (Second Republic)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">1966</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
-        </is>
-      </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zinc</t>
+          <t xml:space="preserve">Vienna (single mint, no mintmark)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Zinc</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">XF (photo estimate)</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Obverse: Austrian federal eagle with hammer, sickle, broken chain, REPUBLIK OSTERREICH. Reverse: large 5, GROSCHEN, edelweiss sprigs. Same year as Coin 9 - duplicate, kept as best grade in that group. Crisp detail.</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">High confidence - date clear</t>
         </is>
@@ -1092,7 +1180,7 @@
         </is>
       </c>
       <c r="B25" s="9">
-        <f>COUNTIF(C5:C20,"5 Groschen")</f>
+        <f>COUNTIF(D5:D20,"5 Groschen")</f>
       </c>
     </row>
     <row r="26">
@@ -1102,7 +1190,7 @@
         </is>
       </c>
       <c r="B26" s="9">
-        <f>COUNTIF(C5:C20,"10 Groschen")</f>
+        <f>COUNTIF(D5:D20,"10 Groschen")</f>
       </c>
     </row>
     <row r="27">
@@ -1112,7 +1200,7 @@
         </is>
       </c>
       <c r="B27" s="9">
-        <f>COUNTIF(C5:C20,"1 Groschen")</f>
+        <f>COUNTIF(D5:D20,"1 Groschen")</f>
       </c>
     </row>
     <row r="28">
@@ -1122,7 +1210,7 @@
         </is>
       </c>
       <c r="B28" s="9">
-        <f>MIN(E5:E20)</f>
+        <f>MIN(F5:F20)</f>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1220,13 @@
         </is>
       </c>
       <c r="B29" s="9">
-        <f>MAX(E5:E20)</f>
+        <f>MAX(F5:F20)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A23:C23"/>
   </mergeCells>
 </worksheet>

</xml_diff>